<commit_message>
WO-REF01-XLS03-FUNCTIONAL-QA-REPAIR-003: 118종 Excel 서식 기능 교정 완결
FIX-A: CHECKLIST ○/× 유효성검사를 결과·여부·유무·확인 열에만 적용
FIX-B: repeat_table → Excel Table (TableStyleMedium2) + max(default×4, 60)행 사전할당
FIX-C: SUM 수식 전면 제거 (의미 검증 실패)
FIX-D: 섹션 JSON 정의 순서 렌더링 + approval 섹션 레벨 label 출력 + xlsx_field_coverage.py 신설
FIX-E: 문서 메타데이터 (title/description/creator) 전체 적용

pytest 188/188 PASS | 유효성검사 118/118 PASS | 필드커버리지 118/118 PASS

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reference-forms/output/xlsx/TAI-FORM-CHW-01.xlsx
+++ b/docs/reference-forms/output/xlsx/TAI-FORM-CHW-01.xlsx
@@ -10,8 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="화학물질 입고·검수 기록표" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'화학물질 입고·검수 기록표'!$A$4:$G$12</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'화학물질 입고·검수 기록표'!$A$1:$G$13</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'화학물질 입고·검수 기록표'!$A$1:$G$266</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -203,6 +202,22 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_CHW_01_1" displayName="T_CHW_01_1" ref="A4:G64" headerRowCount="1">
+  <autoFilter ref="A4:G64"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="제품명"/>
+    <tableColumn id="2" name="제조번호/로트"/>
+    <tableColumn id="3" name="수량"/>
+    <tableColumn id="4" name="용기상태(입력)"/>
+    <tableColumn id="5" name="MSDS버전 확인(입력)"/>
+    <tableColumn id="6" name="이상 내용"/>
+    <tableColumn id="7" name="판정(입력)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -494,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23.4" customWidth="1" min="1" max="1"/>
@@ -650,24 +665,494 @@
       <c r="F12" s="5" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr"/>
     </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="5" t="inlineStr"/>
+      <c r="B13" s="5" t="inlineStr"/>
+      <c r="C13" s="5" t="inlineStr"/>
+      <c r="D13" s="5" t="inlineStr"/>
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr"/>
+      <c r="C14" s="5" t="inlineStr"/>
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="5" t="inlineStr"/>
+      <c r="B15" s="5" t="inlineStr"/>
+      <c r="C15" s="5" t="inlineStr"/>
+      <c r="D15" s="5" t="inlineStr"/>
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="5" t="inlineStr"/>
+      <c r="B16" s="5" t="inlineStr"/>
+      <c r="C16" s="5" t="inlineStr"/>
+      <c r="D16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="5" t="inlineStr"/>
+      <c r="B17" s="5" t="inlineStr"/>
+      <c r="C17" s="5" t="inlineStr"/>
+      <c r="D17" s="5" t="inlineStr"/>
+      <c r="E17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="5" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr"/>
+      <c r="C18" s="5" t="inlineStr"/>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="5" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr"/>
+      <c r="C19" s="5" t="inlineStr"/>
+      <c r="D19" s="5" t="inlineStr"/>
+      <c r="E19" s="5" t="inlineStr"/>
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="5" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr"/>
+      <c r="C20" s="5" t="inlineStr"/>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="5" t="inlineStr"/>
+      <c r="B21" s="5" t="inlineStr"/>
+      <c r="C21" s="5" t="inlineStr"/>
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="5" t="inlineStr"/>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="5" t="inlineStr"/>
+      <c r="B22" s="5" t="inlineStr"/>
+      <c r="C22" s="5" t="inlineStr"/>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="5" t="inlineStr"/>
+      <c r="B23" s="5" t="inlineStr"/>
+      <c r="C23" s="5" t="inlineStr"/>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="5" t="inlineStr"/>
+      <c r="F23" s="5" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="5" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr"/>
+      <c r="C24" s="5" t="inlineStr"/>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="5" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr"/>
+      <c r="C25" s="5" t="inlineStr"/>
+      <c r="D25" s="5" t="inlineStr"/>
+      <c r="E25" s="5" t="inlineStr"/>
+      <c r="F25" s="5" t="inlineStr"/>
+      <c r="G25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="5" t="inlineStr"/>
+      <c r="B26" s="5" t="inlineStr"/>
+      <c r="C26" s="5" t="inlineStr"/>
+      <c r="D26" s="5" t="inlineStr"/>
+      <c r="E26" s="5" t="inlineStr"/>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="5" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr"/>
+      <c r="C27" s="5" t="inlineStr"/>
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="5" t="inlineStr"/>
+      <c r="F27" s="5" t="inlineStr"/>
+      <c r="G27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="5" t="inlineStr"/>
+      <c r="B28" s="5" t="inlineStr"/>
+      <c r="C28" s="5" t="inlineStr"/>
+      <c r="D28" s="5" t="inlineStr"/>
+      <c r="E28" s="5" t="inlineStr"/>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="5" t="inlineStr"/>
+      <c r="B29" s="5" t="inlineStr"/>
+      <c r="C29" s="5" t="inlineStr"/>
+      <c r="D29" s="5" t="inlineStr"/>
+      <c r="E29" s="5" t="inlineStr"/>
+      <c r="F29" s="5" t="inlineStr"/>
+      <c r="G29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="5" t="inlineStr"/>
+      <c r="B30" s="5" t="inlineStr"/>
+      <c r="C30" s="5" t="inlineStr"/>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="5" t="inlineStr"/>
+      <c r="B31" s="5" t="inlineStr"/>
+      <c r="C31" s="5" t="inlineStr"/>
+      <c r="D31" s="5" t="inlineStr"/>
+      <c r="E31" s="5" t="inlineStr"/>
+      <c r="F31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="5" t="inlineStr"/>
+      <c r="B32" s="5" t="inlineStr"/>
+      <c r="C32" s="5" t="inlineStr"/>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="5" t="inlineStr"/>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="5" t="inlineStr"/>
+      <c r="B33" s="5" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr"/>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="5" t="inlineStr"/>
+      <c r="F33" s="5" t="inlineStr"/>
+      <c r="G33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="5" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr"/>
+      <c r="C34" s="5" t="inlineStr"/>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="5" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr"/>
+      <c r="D35" s="5" t="inlineStr"/>
+      <c r="E35" s="5" t="inlineStr"/>
+      <c r="F35" s="5" t="inlineStr"/>
+      <c r="G35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="5" t="inlineStr"/>
+      <c r="B36" s="5" t="inlineStr"/>
+      <c r="C36" s="5" t="inlineStr"/>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="5" t="inlineStr"/>
+      <c r="B37" s="5" t="inlineStr"/>
+      <c r="C37" s="5" t="inlineStr"/>
+      <c r="D37" s="5" t="inlineStr"/>
+      <c r="E37" s="5" t="inlineStr"/>
+      <c r="F37" s="5" t="inlineStr"/>
+      <c r="G37" s="5" t="inlineStr"/>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="5" t="inlineStr"/>
+      <c r="B38" s="5" t="inlineStr"/>
+      <c r="C38" s="5" t="inlineStr"/>
+      <c r="D38" s="5" t="inlineStr"/>
+      <c r="E38" s="5" t="inlineStr"/>
+      <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr"/>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="5" t="inlineStr"/>
+      <c r="B39" s="5" t="inlineStr"/>
+      <c r="C39" s="5" t="inlineStr"/>
+      <c r="D39" s="5" t="inlineStr"/>
+      <c r="E39" s="5" t="inlineStr"/>
+      <c r="F39" s="5" t="inlineStr"/>
+      <c r="G39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="5" t="inlineStr"/>
+      <c r="B40" s="5" t="inlineStr"/>
+      <c r="C40" s="5" t="inlineStr"/>
+      <c r="D40" s="5" t="inlineStr"/>
+      <c r="E40" s="5" t="inlineStr"/>
+      <c r="F40" s="5" t="inlineStr"/>
+      <c r="G40" s="5" t="inlineStr"/>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="5" t="inlineStr"/>
+      <c r="B41" s="5" t="inlineStr"/>
+      <c r="C41" s="5" t="inlineStr"/>
+      <c r="D41" s="5" t="inlineStr"/>
+      <c r="E41" s="5" t="inlineStr"/>
+      <c r="F41" s="5" t="inlineStr"/>
+      <c r="G41" s="5" t="inlineStr"/>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="5" t="inlineStr"/>
+      <c r="B42" s="5" t="inlineStr"/>
+      <c r="C42" s="5" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr"/>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="5" t="inlineStr"/>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="5" t="inlineStr"/>
+      <c r="B43" s="5" t="inlineStr"/>
+      <c r="C43" s="5" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr"/>
+      <c r="F43" s="5" t="inlineStr"/>
+      <c r="G43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="5" t="inlineStr"/>
+      <c r="B44" s="5" t="inlineStr"/>
+      <c r="C44" s="5" t="inlineStr"/>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="5" t="inlineStr"/>
+      <c r="B45" s="5" t="inlineStr"/>
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr"/>
+      <c r="E45" s="5" t="inlineStr"/>
+      <c r="F45" s="5" t="inlineStr"/>
+      <c r="G45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="5" t="inlineStr"/>
+      <c r="B46" s="5" t="inlineStr"/>
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr"/>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="A47" s="5" t="inlineStr"/>
+      <c r="B47" s="5" t="inlineStr"/>
+      <c r="C47" s="5" t="inlineStr"/>
+      <c r="D47" s="5" t="inlineStr"/>
+      <c r="E47" s="5" t="inlineStr"/>
+      <c r="F47" s="5" t="inlineStr"/>
+      <c r="G47" s="5" t="inlineStr"/>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="5" t="inlineStr"/>
+      <c r="B48" s="5" t="inlineStr"/>
+      <c r="C48" s="5" t="inlineStr"/>
+      <c r="D48" s="5" t="inlineStr"/>
+      <c r="E48" s="5" t="inlineStr"/>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="5" t="inlineStr"/>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="5" t="inlineStr"/>
+      <c r="B49" s="5" t="inlineStr"/>
+      <c r="C49" s="5" t="inlineStr"/>
+      <c r="D49" s="5" t="inlineStr"/>
+      <c r="E49" s="5" t="inlineStr"/>
+      <c r="F49" s="5" t="inlineStr"/>
+      <c r="G49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="5" t="inlineStr"/>
+      <c r="B50" s="5" t="inlineStr"/>
+      <c r="C50" s="5" t="inlineStr"/>
+      <c r="D50" s="5" t="inlineStr"/>
+      <c r="E50" s="5" t="inlineStr"/>
+      <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="5" t="inlineStr"/>
+    </row>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="5" t="inlineStr"/>
+      <c r="B51" s="5" t="inlineStr"/>
+      <c r="C51" s="5" t="inlineStr"/>
+      <c r="D51" s="5" t="inlineStr"/>
+      <c r="E51" s="5" t="inlineStr"/>
+      <c r="F51" s="5" t="inlineStr"/>
+      <c r="G51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="5" t="inlineStr"/>
+      <c r="B52" s="5" t="inlineStr"/>
+      <c r="C52" s="5" t="inlineStr"/>
+      <c r="D52" s="5" t="inlineStr"/>
+      <c r="E52" s="5" t="inlineStr"/>
+      <c r="F52" s="5" t="inlineStr"/>
+      <c r="G52" s="5" t="inlineStr"/>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="5" t="inlineStr"/>
+      <c r="B53" s="5" t="inlineStr"/>
+      <c r="C53" s="5" t="inlineStr"/>
+      <c r="D53" s="5" t="inlineStr"/>
+      <c r="E53" s="5" t="inlineStr"/>
+      <c r="F53" s="5" t="inlineStr"/>
+      <c r="G53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="5" t="inlineStr"/>
+      <c r="B54" s="5" t="inlineStr"/>
+      <c r="C54" s="5" t="inlineStr"/>
+      <c r="D54" s="5" t="inlineStr"/>
+      <c r="E54" s="5" t="inlineStr"/>
+      <c r="F54" s="5" t="inlineStr"/>
+      <c r="G54" s="5" t="inlineStr"/>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="5" t="inlineStr"/>
+      <c r="B55" s="5" t="inlineStr"/>
+      <c r="C55" s="5" t="inlineStr"/>
+      <c r="D55" s="5" t="inlineStr"/>
+      <c r="E55" s="5" t="inlineStr"/>
+      <c r="F55" s="5" t="inlineStr"/>
+      <c r="G55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="5" t="inlineStr"/>
+      <c r="B56" s="5" t="inlineStr"/>
+      <c r="C56" s="5" t="inlineStr"/>
+      <c r="D56" s="5" t="inlineStr"/>
+      <c r="E56" s="5" t="inlineStr"/>
+      <c r="F56" s="5" t="inlineStr"/>
+      <c r="G56" s="5" t="inlineStr"/>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="5" t="inlineStr"/>
+      <c r="B57" s="5" t="inlineStr"/>
+      <c r="C57" s="5" t="inlineStr"/>
+      <c r="D57" s="5" t="inlineStr"/>
+      <c r="E57" s="5" t="inlineStr"/>
+      <c r="F57" s="5" t="inlineStr"/>
+      <c r="G57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58" ht="16" customHeight="1">
+      <c r="A58" s="5" t="inlineStr"/>
+      <c r="B58" s="5" t="inlineStr"/>
+      <c r="C58" s="5" t="inlineStr"/>
+      <c r="D58" s="5" t="inlineStr"/>
+      <c r="E58" s="5" t="inlineStr"/>
+      <c r="F58" s="5" t="inlineStr"/>
+      <c r="G58" s="5" t="inlineStr"/>
+    </row>
+    <row r="59" ht="16" customHeight="1">
+      <c r="A59" s="5" t="inlineStr"/>
+      <c r="B59" s="5" t="inlineStr"/>
+      <c r="C59" s="5" t="inlineStr"/>
+      <c r="D59" s="5" t="inlineStr"/>
+      <c r="E59" s="5" t="inlineStr"/>
+      <c r="F59" s="5" t="inlineStr"/>
+      <c r="G59" s="5" t="inlineStr"/>
+    </row>
+    <row r="60" ht="16" customHeight="1">
+      <c r="A60" s="5" t="inlineStr"/>
+      <c r="B60" s="5" t="inlineStr"/>
+      <c r="C60" s="5" t="inlineStr"/>
+      <c r="D60" s="5" t="inlineStr"/>
+      <c r="E60" s="5" t="inlineStr"/>
+      <c r="F60" s="5" t="inlineStr"/>
+      <c r="G60" s="5" t="inlineStr"/>
+    </row>
+    <row r="61" ht="16" customHeight="1">
+      <c r="A61" s="5" t="inlineStr"/>
+      <c r="B61" s="5" t="inlineStr"/>
+      <c r="C61" s="5" t="inlineStr"/>
+      <c r="D61" s="5" t="inlineStr"/>
+      <c r="E61" s="5" t="inlineStr"/>
+      <c r="F61" s="5" t="inlineStr"/>
+      <c r="G61" s="5" t="inlineStr"/>
+    </row>
+    <row r="62" ht="16" customHeight="1">
+      <c r="A62" s="5" t="inlineStr"/>
+      <c r="B62" s="5" t="inlineStr"/>
+      <c r="C62" s="5" t="inlineStr"/>
+      <c r="D62" s="5" t="inlineStr"/>
+      <c r="E62" s="5" t="inlineStr"/>
+      <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="5" t="inlineStr"/>
+    </row>
+    <row r="63" ht="16" customHeight="1">
+      <c r="A63" s="5" t="inlineStr"/>
+      <c r="B63" s="5" t="inlineStr"/>
+      <c r="C63" s="5" t="inlineStr"/>
+      <c r="D63" s="5" t="inlineStr"/>
+      <c r="E63" s="5" t="inlineStr"/>
+      <c r="F63" s="5" t="inlineStr"/>
+      <c r="G63" s="5" t="inlineStr"/>
+    </row>
+    <row r="64" ht="16" customHeight="1">
+      <c r="A64" s="5" t="inlineStr"/>
+      <c r="B64" s="5" t="inlineStr"/>
+      <c r="C64" s="5" t="inlineStr"/>
+      <c r="D64" s="5" t="inlineStr"/>
+      <c r="E64" s="5" t="inlineStr"/>
+      <c r="F64" s="5" t="inlineStr"/>
+      <c r="G64" s="5" t="inlineStr"/>
+    </row>
+    <row r="65" ht="28" customHeight="1">
+      <c r="A65" s="6" t="inlineStr">
         <is>
           <t>【입력 안내】 용기상태·MSDS버전 확인란은 사업장 기준에 따라 직접 기재하십시오. 판정란에는 합격·격리·반품 등 사업장 기준에 따라 기재하십시오. 이 서식은 법정 검수 절차를 확인한 것이 아닙니다.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G12"/>
   <mergeCells count="6">
-    <mergeCell ref="A13:G13"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="E3:G3"/>
+    <mergeCell ref="A65:G65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>